<commit_message>
feat(F-NAR-019): ATOM-EMO.LEX.003-08 Le citron de Victorina
</commit_message>
<xml_diff>
--- a/stories/arbres/ATOM-EMO.LEX.003-08.xlsx
+++ b/stories/arbres/ATOM-EMO.LEX.003-08.xlsx
@@ -671,7 +671,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>marché</t>
+          <t>marché, barquette, basilic, citron, fraises, panier, table, herbes, linge, plastique, verre</t>
         </is>
       </c>
     </row>
@@ -683,7 +683,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Victorina, maman</t>
+          <t>Victorina, papa, maman</t>
         </is>
       </c>
     </row>
@@ -841,7 +841,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Victorina veut les fraises. C'est pour plus tard. Elle dit qu'elle est déçue. Elle sent le basilic. Elle choisit un citron.</t>
+          <t>Une tige de basilic accroche la manche. Sur le plastique, un éclat de barquette luit. Victorina veut les fraises, maintenant. Les fraises, c'est pour plus tard. Sourire parti. Trou dans la poitrine. Papa s'accroupit. Je suis déçue. Merci vécu. Elle sent le basilic. Deuxième ruse : basilic qui glisse, citron trop acide. Elle refuse de foncer. Elle choisit un citron. Un éclat de barquette tient.</t>
         </is>
       </c>
     </row>
@@ -1184,17 +1184,17 @@
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>La balance du marché fait tic. Un poids tombe, tout léger. Un citron roule sous une caisse. Il s'arrête contre une botte. Le basilic attend dans l'eau. Les feuilles sont vertes et brillantes. Un linge blanc cache des fruits. Le linge sent le soleil. Des oignons violets sentent fort. Tu as entendu la balance, Victorina ? Elle fait tic. C'est le poids. On reste près de moi. Tu tiens bien le panier ? En ce moment, Victorina tient le panier. Le panier gratte un peu la main. Le linge se soulève. Des fraises rouges apparaissent. Les rouges, maman. Les fraises, c'est pour plus tard. Victorina sent sa gorge serrée. Ses épaules descendent. Je suis déçue. Tu es déçue. Je t'écoute. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Victorina souffle une fois. L'air sent les herbes. On sent le basilic ? Une autre idée. Bravo, Victorina. Elles froissent une feuille. Ça sent le vert, tout fort. Ça pique un peu le nez. Oui. Je suis déçue. Et j'ai une autre idée. Victorina regarde le citron arrêté. Celui-là. Le citron. Tu as proposé autre chose. Le citron est lisse et frais. Victorina le pose dans le panier. Il roule, puis il tient. Le souhait peut attendre. Une autre idée, c'est possible. Il est froid. Oui. Comme une petite lune. La balance fait encore tic, plus loin. Le basilic tremble dans l'eau.</t>
+          <t>Une tige de basilic accroche la manche de Victorina. Elle pique, papa ! Tu la vois, la tige ? Oui, papa. Papa détache la tige, près du panier. Elle sent le vert. Tu la sens, Victorina ? Oui, maman. Le marché sent les herbes, près des tables. Ça sent fort. Tu le sens, le vert ? Oui, papa. Ils avancent vers le passage des herbes. Des feuilles dans l'eau. Tu les vois, les vertes ? Oui, maman. Le basilic tremble dans un verre d'eau. Il tremble. Tu le vois, le basilic ? Oui, papa. Une barquette de fraises attend, près du verre. Des rouges ! Tu les vois, les fraises ? Oui, maman. Sur le plastique, un éclat de barquette luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le plastique de la barquette est un peu froid. Il est froid. Tes doigts sont bien, Victorina ? Un peu froids. Un linge blanc cache d'autres fruits, plus loin. Il sent le soleil. Tu le sens, le linge ? Oui, papa. En ce moment, Victorina tend les deux mains. Je veux les fraises, maintenant ! Tout de suite ? Oui, papa. Victorina avance trop vite vers la barquette. Ses doigts touchent seulement le plastique. Les fraises, c'est pour plus tard. Maintenant ! Les rouges restent dans la barquette. Je les veux. Plus tard, Victorina ? Non, maman. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie des fraises fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Victorina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Victorina ? Un peu, maman. Je suis déçue. L'éclat de barquette tremble, puis tient. Victorina lève les yeux vers les herbes. Du basilic. Tu le vois, Victorina ? Oui, papa. Le panier reste près de toi ? Oui, maman.</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>La balance du marché fait tic. Un poids tombe, tout léger. Un citron roule sous une caisse. Il s'arrête contre une botte. Le basilic attend dans l'eau. Les feuilles sont vertes et brillantes. Un linge blanc cache des fruits. Le linge sent le soleil. Des oignons violets sentent fort. Tu as entendu la balance, Victorina ? Elle fait tic. C'est le poids. On reste près de moi. Tu tiens bien le panier ? En ce moment, Victorina tient le panier. Le panier gratte un peu la main. Le linge se soulève. Des fraises rouges apparaissent. Les rouges, maman. Les fraises, c'est pour plus tard. Victorina sent sa gorge serrée. Ses épaules descendent. Je suis déçue. Tu es déçue. Je t'écoute. Ce n'est pas honteux. Un souhait peut attendre. On peut chercher une autre idée. Victorina souffle une fois. L'air sent les herbes. On sent le basilic ? Une autre idée. Bravo, Victorina. Elles froissent une feuille. Ça sent le vert, tout fort. Ça pique un peu le nez. Oui. Je suis déçue. Et j'ai une autre idée. Victorina regarde le citron arrêté. Celui-là. Le citron. Tu as proposé autre chose. Le citron est lisse et frais. Victorina le pose dans le panier. Il roule, puis il tient. Le souhait peut attendre. Une autre idée, c'est possible. Il est froid. Oui. Comme une petite lune. La balance fait encore tic, plus loin. Le basilic tremble dans l'eau.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Une tige de basilic accroche la manche de Victorina. Elle pique, papa ! Tu la vois, la tige ? Oui, papa. Papa détache la tige, près du panier. Elle sent le vert. Tu la sens, Victorina ? Oui, maman. Le marché sent les herbes, près des tables. Ça sent fort. Tu le sens, le vert ? Oui, papa. Ils avancent vers le passage des herbes. Des feuilles dans l'eau. Tu les vois, les vertes ? Oui, maman. Le basilic tremble dans un verre d'eau. Il tremble. Tu le vois, le basilic ? Oui, papa. Une barquette de fraises attend, près du verre. Des rouges ! Tu les vois, les fraises ? Oui, maman. Sur le plastique, un &lt;emphasis level="moderate"&gt;éclat de barquette&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le plastique de la barquette est un peu froid. Il est froid. Tes doigts sont bien, Victorina ? Un peu froids. Un linge blanc cache d'autres fruits, plus loin. Il sent le soleil. Tu le sens, le linge ? Oui, papa. En ce moment, Victorina tend les deux mains. Je veux les fraises, maintenant ! Tout de suite ? Oui, papa. Victorina avance trop vite vers la barquette. Ses doigts touchent seulement le plastique. Les fraises, c'est pour plus tard. Maintenant ! Les rouges restent dans la barquette. Je les veux. Plus tard, Victorina ? Non, maman. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie des fraises fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Victorina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Victorina ? Un peu, maman. Je suis déçue. L'éclat de barquette tremble, puis tient. Victorina lève les yeux vers les herbes. Du basilic. Tu le vois, Victorina ? Oui, papa. Le panier reste près de toi ? Oui, maman.&lt;/prosody&gt;&lt;break time="500ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>Geneviève est au marché avec maman. Elle voit des fraises rouges. Elle a envie. Maman dit : les fraises, c'est pour plus tard. Geneviève sent sa gorge serrée. Ses épaules descendent. Elle dit : je suis &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Maman écoute. Maman dit : on peut chercher une autre idée. Geneviève respire. Elle propose : on sent le basilic. Elles froissent une feuille. Ça sent le vert. Geneviève dit encore : je suis déçue. Et j'ai une autre idée. Elle choisit un citron. Le citron est lisse et frais. Maman sourit. Geneviève pose le citron dans le panier. Le souhait peut attendre. Une autre idée, c'est possible. [pause]</t>
+          <t>Une tige de basilic accroche la manche de Victorina. Elle pique, papa ! Tu la vois, la tige ? Oui, papa. Papa détache la tige, près du panier. Elle sent le vert. Tu la sens, Victorina ? Oui, maman. Le marché sent les herbes, près des tables. Ça sent fort. Tu le sens, le vert ? Oui, papa. Ils avancent vers le passage des herbes. Des feuilles dans l'eau. Tu les vois, les vertes ? Oui, maman. Le basilic tremble dans un verre d'eau. Il tremble. Tu le vois, le basilic ? Oui, papa. Une barquette de fraises attend, près du verre. Des rouges ! Tu les vois, les fraises ? Oui, maman. Sur le plastique, un &lt;emphasis&gt;éclat de barquette&lt;/emphasis&gt; luit. Il brille, papa. Tu le vois, le petit point ? Oui, un point clair. Le plastique de la barquette est un peu froid. Il est froid. Tes doigts sont bien, Victorina ? Un peu froids. Un linge blanc cache d'autres fruits, plus loin. Il sent le soleil. Tu le sens, le linge ? Oui, papa. En ce moment, Victorina tend les deux mains. Je veux les fraises, maintenant ! Tout de suite ? Oui, papa. Victorina avance trop vite vers la barquette. Ses doigts touchent seulement le plastique. Les fraises, c'est pour plus tard. Maintenant ! Les rouges restent dans la barquette. Je les veux. Plus tard, Victorina ? Non, maman. Le sourire de Victorina disparaît. Dans sa poitrine, l'envie des fraises fait un trou. L'envie et le trou se bousculent sans place. Ses épaules tombent un peu. J'ai mal au ventre. Ta gorge est serrée, Victorina ? Un peu, papa. Papa s'accroupit à la même hauteur, sans parler. Tes mains sont chaudes, Victorina ? Un peu, maman. Je suis déçue. L'éclat de barquette tremble, puis tient. Victorina lève les yeux vers les herbes. Du basilic. Tu le vois, Victorina ? Oui, papa. Le panier reste près de toi ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr"/>
@@ -1241,7 +1241,7 @@
         </is>
       </c>
       <c r="Y2" s="2" t="n">
-        <v>132</v>
+        <v>142</v>
       </c>
       <c r="Z2" s="2" t="inlineStr">
         <is>
@@ -1249,10 +1249,10 @@
         </is>
       </c>
       <c r="AA2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AB2" s="2" t="n">
-        <v>1.18</v>
+        <v>1.12</v>
       </c>
       <c r="AC2" s="2" t="inlineStr">
         <is>
@@ -1275,30 +1275,30 @@
       </c>
       <c r="AH2" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>éclat de barquette</t>
         </is>
       </c>
       <c r="AI2" s="2" t="n">
         <v>0</v>
       </c>
       <c r="AJ2" s="2" t="n">
-        <v>400</v>
+        <v>500</v>
       </c>
       <c r="AK2" s="2" t="n">
-        <v>280</v>
+        <v>260</v>
       </c>
       <c r="AL2" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>warm</t>
         </is>
       </c>
       <c r="AM2" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>storytelling</t>
         </is>
       </c>
       <c r="AN2" s="2" t="n">
-        <v>0.333</v>
+        <v>0.36</v>
       </c>
       <c r="AO2" s="2" t="inlineStr"/>
       <c r="AP2" s="2" t="inlineStr">
@@ -1307,10 +1307,10 @@
         </is>
       </c>
       <c r="AQ2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AR2" s="2" t="n">
-        <v>0.92</v>
+        <v>0.98</v>
       </c>
       <c r="AS2" s="2" t="n">
         <v>100</v>
@@ -1321,62 +1321,84 @@
       <c r="AU2" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV2" s="2" t="inlineStr"/>
+      <c r="AV2" s="2" t="inlineStr">
+        <is>
+          <t>arc=installation; intention=émerveiller puis tendre; emotion=impatience puis déception; intensite=2; destinataire=enfant; sous_texte=elle_veut_les_fraises_maintenant; tempo=naturel puis resserré; sourire=léger puis aucun; respiration=ample puis retenue</t>
+        </is>
+      </c>
       <c r="AW2" t="inlineStr">
         <is>
-          <t>narrateur|La balance du marché fait tic.
-narrateur|Un poids tombe, tout léger.
-narrateur|Un citron roule sous une caisse.
-narrateur|Il s'arrête contre une botte.
-narrateur|Le basilic attend dans l'eau.
-narrateur|Les feuilles sont vertes et brillantes.
-narrateur|Un linge blanc cache des fruits.
-narrateur|Le linge sent le soleil.
-narrateur|Des oignons violets sentent fort.
-maman|Tu as entendu la balance, Victorina ?
-enfant-f|Elle fait tic.
-maman|C'est le poids.
-maman|On reste près de moi.
-maman|Tu tiens bien le panier ?
-narrateur|En ce moment, Victorina tient le panier.
-narrateur|Le panier gratte un peu la main.
-narrateur|Le linge se soulève.
-narrateur|Des fraises rouges apparaissent.
-enfant-f|Les rouges, maman.
+          <t>narrateur|Une tige de basilic accroche la manche de Victorina.
+enfant-f|Elle pique, papa !
+papa|Tu la vois, la tige ?
+enfant-f|Oui, papa.
+narrateur|Papa détache la tige, près du panier.
+enfant-f|Elle sent le vert.
+maman|Tu la sens, Victorina ?
+enfant-f|Oui, maman.
+narrateur|Le marché sent les herbes, près des tables.
+enfant-f|Ça sent fort.
+papa|Tu le sens, le vert ?
+enfant-f|Oui, papa.
+narrateur|Ils avancent vers le passage des herbes.
+enfant-f|Des feuilles dans l'eau.
+maman|Tu les vois, les vertes ?
+enfant-f|Oui, maman.
+narrateur|Le basilic tremble dans un verre d'eau.
+enfant-f|Il tremble.
+papa|Tu le vois, le basilic ?
+enfant-f|Oui, papa.
+narrateur|Une barquette de fraises attend, près du verre.
+enfant-f|Des rouges !
+maman|Tu les vois, les fraises ?
+enfant-f|Oui, maman.
+narrateur|Sur le plastique, un éclat de barquette luit.
+enfant-f|Il brille, papa.
+papa|Tu le vois, le petit point ?
+enfant-f|Oui, un point clair.
+narrateur|Le plastique de la barquette est un peu froid.
+enfant-f|Il est froid.
+maman|Tes doigts sont bien, Victorina ?
+enfant-f|Un peu froids.
+narrateur|Un linge blanc cache d'autres fruits, plus loin.
+enfant-f|Il sent le soleil.
+papa|Tu le sens, le linge ?
+enfant-f|Oui, papa.
+narrateur|En ce moment, Victorina tend les deux mains.
+enfant-f|Je veux les fraises, maintenant !
+papa|Tout de suite ?
+enfant-f|Oui, papa.
+narrateur|Victorina avance trop vite vers la barquette.
+narrateur|Ses doigts touchent seulement le plastique.
 maman|Les fraises, c'est pour plus tard.
-narrateur|Victorina sent sa gorge serrée.
-narrateur|Ses épaules descendent.
+enfant-f|Maintenant !
+narrateur|Les rouges restent dans la barquette.
+enfant-f|Je les veux.
+maman|Plus tard, Victorina ?
+enfant-f|Non, maman.
+narrateur|Le sourire de Victorina disparaît.
+narrateur|Dans sa poitrine, l'envie des fraises fait un trou.
+narrateur|L'envie et le trou se bousculent sans place.
+narrateur|Ses épaules tombent un peu.
+enfant-f|J'ai mal au ventre.
+papa|Ta gorge est serrée, Victorina ?
+enfant-f|Un peu, papa.
+narrateur|Papa s'accroupit à la même hauteur, sans parler.
+maman|Tes mains sont chaudes, Victorina ?
+enfant-f|Un peu, maman.
 enfant-f|Je suis déçue.
-maman|Tu es déçue.
-maman|Je t'écoute.
-maman|Ce n'est pas honteux.
-maman|Un souhait peut attendre.
-maman|On peut chercher une autre idée.
-narrateur|Victorina souffle une fois.
-narrateur|L'air sent les herbes.
-enfant-f|On sent le basilic ?
-maman|Une autre idée.
-maman|Bravo, Victorina.
-narrateur|Elles froissent une feuille.
-narrateur|Ça sent le vert, tout fort.
-enfant-f|Ça pique un peu le nez.
-maman|Oui.
-enfant-f|Je suis déçue.
-enfant-f|Et j'ai une autre idée.
-narrateur|Victorina regarde le citron arrêté.
-enfant-f|Celui-là.
-maman|Le citron.
-maman|Tu as proposé autre chose.
-narrateur|Le citron est lisse et frais.
-narrateur|Victorina le pose dans le panier.
-narrateur|Il roule, puis il tient.
-maman|Le souhait peut attendre.
-maman|Une autre idée, c'est possible.
-enfant-f|Il est froid.
-maman|Oui.
-maman|Comme une petite lune.
-narrateur|La balance fait encore tic, plus loin.
-narrateur|Le basilic tremble dans l'eau.</t>
+narrateur|L'éclat de barquette tremble, puis tient.
+narrateur|Victorina lève les yeux vers les herbes.
+enfant-f|Du basilic.
+papa|Tu le vois, Victorina ?
+enfant-f|Oui, papa.
+maman|Le panier reste près de toi ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX2" t="inlineStr">
+        <is>
+          <t>marché,basilic</t>
         </is>
       </c>
     </row>
@@ -1408,12 +1430,12 @@
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>Victorina n'a pas les fraises. Que dit-elle ?</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="medium"&gt;&lt;emphasis level="moderate"&gt;Victorina&lt;/emphasis&gt; n'a pas les fraises. Que dit-elle ?&lt;/prosody&gt;&lt;break time="700ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>&lt;slow&gt;Geneviève n'a pas les fraises. Que dit-elle ?&lt;/slow&gt;</t>
+          <t>&lt;soft&gt;&lt;slow&gt;&lt;emphasis&gt;Victorina&lt;/emphasis&gt; n'a pas les fraises. Que dit-elle ?&lt;/slow&gt;&lt;/soft&gt; [pause]</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
@@ -1476,7 +1498,7 @@
         </is>
       </c>
       <c r="Y3" s="2" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
       <c r="Z3" s="2" t="inlineStr">
         <is>
@@ -1487,7 +1509,7 @@
         <v>0.86</v>
       </c>
       <c r="AB3" s="2" t="n">
-        <v>1.3</v>
+        <v>1.27</v>
       </c>
       <c r="AC3" s="2" t="inlineStr">
         <is>
@@ -1502,34 +1524,38 @@
       <c r="AE3" s="2" t="inlineStr"/>
       <c r="AF3" s="2" t="inlineStr">
         <is>
-          <t>medium</t>
+          <t>soft</t>
         </is>
       </c>
       <c r="AG3" s="2" t="n">
-        <v>0</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr"/>
+        <v>-2</v>
+      </c>
+      <c r="AH3" s="2" t="inlineStr">
+        <is>
+          <t>Victorina</t>
+        </is>
+      </c>
       <c r="AI3" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ3" s="2" t="n">
-        <v>250</v>
+        <v>700</v>
       </c>
       <c r="AK3" s="2" t="n">
-        <v>280</v>
+        <v>320</v>
       </c>
       <c r="AL3" s="2" t="inlineStr">
         <is>
-          <t>warm</t>
+          <t>focused</t>
         </is>
       </c>
       <c r="AM3" s="2" t="inlineStr">
         <is>
-          <t>rise</t>
+          <t>rising</t>
         </is>
       </c>
       <c r="AN3" s="2" t="n">
-        <v>0.333</v>
+        <v>0.32</v>
       </c>
       <c r="AO3" s="2" t="inlineStr"/>
       <c r="AP3" s="2" t="inlineStr">
@@ -1544,17 +1570,17 @@
         <v>0.86</v>
       </c>
       <c r="AS3" s="2" t="n">
-        <v>100</v>
+        <v>82</v>
       </c>
       <c r="AT3" s="2" t="n">
         <v>50</v>
       </c>
       <c r="AU3" s="2" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="AV3" s="2" t="inlineStr">
         <is>
-          <t>question d'écoute, ne change pas le cours</t>
+          <t>arc=indice; intention=faire_deviner; emotion=attention; intensite=1; destinataire=enfant; sous_texte=elle_n_a_pas_les_fraises_que_dit_elle; tempo=suspendu; sourire=aucun; respiration=courte_avant_question</t>
         </is>
       </c>
       <c r="AW3" t="inlineStr">
@@ -1587,17 +1613,17 @@
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Victorina touche encore le citron. J'ai dit : je suis déçue. Oui. Tu as nommé. Puis une autre idée. Le basilic, puis le citron. Bravo, Victorina. Le souhait peut attendre. Oui. Le panier gratte encore un peu.</t>
+          <t>Victorina reste près de la barquette, un moment. Les fraises, maintenant. Les mots se bousculent dans sa bouche. Je les prends. Victorina avance les mains, trop vite. Puis elle s'arrête. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les herbes, un instant. Elle écoute le marché, près des tables. Tu restes un peu, Victorina ? Oui, papa. Merci, Victorina. Papa reste à la même hauteur. Le basilic sent fort, sous les doigts. Il est mouillé. La poitrine de Victorina ralentit un peu. Les épaules se relèvent un peu. On sent le basilic ? Tu la froisses, la feuille ? Oui, maman. Ça sent le vert, Victorina ? Ça pique un peu le nez. Victorina froisse une feuille, sans se presser. Le vert, papa. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. Le basilic, papa. On y va, sans se presser. Un citron, aussi. Tu le vois, le jaune ? Oui, maman.</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>Victorina touche encore le citron. J'ai dit : je suis déçue. Oui. Tu as nommé. Puis une autre idée. Le basilic, puis le citron. Bravo, Victorina. Le souhait peut attendre. Oui. Le panier gratte encore un peu.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina reste près de la barquette, un moment. Les fraises, maintenant. Les mots se bousculent dans sa bouche. Je les prends. Victorina avance les mains, trop vite. Puis elle s'arrête. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les herbes, un instant. Elle écoute le marché, près des tables. Tu restes un peu, Victorina ? Oui, papa. Merci, Victorina. Papa reste à la même hauteur. Le &lt;emphasis level="moderate"&gt;basilic&lt;/emphasis&gt; sent fort, sous les doigts. Il est mouillé. La poitrine de Victorina ralentit un peu. Les épaules se relèvent un peu. On sent le basilic ? Tu la froisses, la feuille ? Oui, maman. Ça sent le vert, Victorina ? Ça pique un peu le nez. Victorina froisse une feuille, sans se presser. Le vert, papa. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. Le basilic, papa. On y va, sans se presser. Un citron, aussi. Tu le vois, le jaune ? Oui, maman.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>Geneviève a nommé. Elle était &lt;emphasis&gt;déçu&lt;/emphasis&gt;e. Elle a trouvé une autre idée. Maman était là. [pause]</t>
+          <t>Victorina reste près de la barquette, un moment. Les fraises, maintenant. Les mots se bousculent dans sa bouche. Je les prends. Victorina avance les mains, trop vite. Puis elle s'arrête. Victorina refuse de foncer. Elle referme la bouche. Personne ne parle. Elle observe les herbes, un instant. Elle écoute le marché, près des tables. Tu restes un peu, Victorina ? Oui, papa. Merci, Victorina. Papa reste à la même hauteur. Le &lt;emphasis&gt;basilic&lt;/emphasis&gt; sent fort, sous les doigts. Il est mouillé. La poitrine de Victorina ralentit un peu. Les épaules se relèvent un peu. On sent le basilic ? Tu la froisses, la feuille ? Oui, maman. Ça sent le vert, Victorina ? Ça pique un peu le nez. Victorina froisse une feuille, sans se presser. Le vert, papa. On s'approche sans se presser ? Oui. Ils se lèvent, sans se bousculer. Le basilic, papa. On y va, sans se presser. Un citron, aussi. Tu le vois, le jaune ? Oui, maman. [pause]</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr"/>
@@ -1644,7 +1670,7 @@
         </is>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>132</v>
+        <v>140</v>
       </c>
       <c r="Z4" s="2" t="inlineStr">
         <is>
@@ -1652,10 +1678,10 @@
         </is>
       </c>
       <c r="AA4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AB4" s="2" t="n">
-        <v>1.18</v>
+        <v>1.14</v>
       </c>
       <c r="AC4" s="2" t="inlineStr">
         <is>
@@ -1678,30 +1704,30 @@
       </c>
       <c r="AH4" s="2" t="inlineStr">
         <is>
-          <t>déçu</t>
+          <t>basilic</t>
         </is>
       </c>
       <c r="AI4" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ4" s="2" t="n">
-        <v>450</v>
+        <v>560</v>
       </c>
       <c r="AK4" s="2" t="n">
-        <v>280</v>
+        <v>270</v>
       </c>
       <c r="AL4" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>bright</t>
         </is>
       </c>
       <c r="AM4" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN4" s="2" t="n">
-        <v>0.333</v>
+        <v>0.35</v>
       </c>
       <c r="AO4" s="2" t="inlineStr"/>
       <c r="AP4" s="2" t="inlineStr">
@@ -1710,10 +1736,10 @@
         </is>
       </c>
       <c r="AQ4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AR4" s="2" t="n">
-        <v>0.92</v>
+        <v>0.97</v>
       </c>
       <c r="AS4" s="2" t="n">
         <v>100</v>
@@ -1726,21 +1752,50 @@
       </c>
       <c r="AV4" s="2" t="inlineStr">
         <is>
-          <t>confirmation ; le moteur peut dire engine_ok/near avant ce chunk</t>
+          <t>arc=résolution; intention=faire_vivre_le_geste; emotion=retenue puis soulagement; intensite=2; destinataire=enfant; sous_texte=elle_sent_le_basilic_sans_slogan; tempo=naturel; sourire=léger; respiration=relâchée</t>
         </is>
       </c>
       <c r="AW4" t="inlineStr">
         <is>
-          <t>narrateur|Victorina touche encore le citron.
-enfant-f|J'ai dit : je suis déçue.
-maman|Oui.
-maman|Tu as nommé.
-maman|Puis une autre idée.
-maman|Le basilic, puis le citron.
-maman|Bravo, Victorina.
-enfant-f|Le souhait peut attendre.
-maman|Oui.
-narrateur|Le panier gratte encore un peu.</t>
+          <t>narrateur|Victorina reste près de la barquette, un moment.
+enfant-f|Les fraises, maintenant.
+narrateur|Les mots se bousculent dans sa bouche.
+enfant-f|Je les prends.
+narrateur|Victorina avance les mains, trop vite.
+narrateur|Puis elle s'arrête.
+narrateur|Victorina refuse de foncer.
+narrateur|Elle referme la bouche.
+narrateur|Personne ne parle.
+narrateur|Elle observe les herbes, un instant.
+narrateur|Elle écoute le marché, près des tables.
+papa|Tu restes un peu, Victorina ?
+enfant-f|Oui, papa.
+papa|Merci, Victorina.
+narrateur|Papa reste à la même hauteur.
+maman|Le basilic sent fort, sous les doigts.
+enfant-f|Il est mouillé.
+narrateur|La poitrine de Victorina ralentit un peu.
+narrateur|Les épaules se relèvent un peu.
+enfant-f|On sent le basilic ?
+maman|Tu la froisses, la feuille ?
+enfant-f|Oui, maman.
+papa|Ça sent le vert, Victorina ?
+enfant-f|Ça pique un peu le nez.
+narrateur|Victorina froisse une feuille, sans se presser.
+enfant-f|Le vert, papa.
+papa|On s'approche sans se presser ?
+enfant-f|Oui.
+narrateur|Ils se lèvent, sans se bousculer.
+enfant-f|Le basilic, papa.
+papa|On y va, sans se presser.
+enfant-f|Un citron, aussi.
+maman|Tu le vois, le jaune ?
+enfant-f|Oui, maman.</t>
+        </is>
+      </c>
+      <c r="AX4" t="inlineStr">
+        <is>
+          <t>marché</t>
         </is>
       </c>
     </row>
@@ -1767,17 +1822,17 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Victorina tient le citron. Maman porte le panier. On rentre tout doucement ? Oui, maman. Tu as nommé : déçue. Puis tu as cherché. Le citron reste frais dans sa main. Une feuille de basilic sent encore. Il est lisse. Oui. Avec l'autre idée.</t>
+          <t>Victorina lève la main vers le basilic. Je le prends ! La tige glisse entre ses doigts, trop mouillée. Il part ! Le basilic retombe dans l'eau, près du verre. Victorina avance les mains, trop vite. Un citron, alors ! Elle porte un citron trop près du nez. Le citron pique trop, trop acide. Il pique ! Victorina avance trop vite vers le jaune. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le citron, un instant. Elle écoute le marché, près de la barquette. Sur le plastique, un éclat de barquette luit. Là, sur le plastique. Tu vois le point, Victorina ? Oui, papa. Le premier citron reste trop acide, trop près. Pas celui-là. Tu en vois un autre, Victorina ? Plus rond. Un citron plus rond attend à hauteur de main. Celui-là, maman. Tu le prends, Victorina ? Oui, papa. Victorina choisit le citron plus rond, sans se presser. La peau est lisse et froide. Il est lourd. Il tient dans ta main ? Oui, maman. Victorina le pose dans le panier. Mon citron. Il a une petite trace, Victorina. Il a failli piquer. Le citron sent le vert, un peu. Et le basilic, autour. On reste près de la barquette ? Oui.</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>Victorina tient le citron. Maman porte le panier. On rentre tout doucement ? Oui, maman. Tu as nommé : déçue. Puis tu as cherché. Le citron reste frais dans sa main. Une feuille de basilic sent encore. Il est lisse. Oui. Avec l'autre idée.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Victorina lève la main vers le basilic. Je le prends ! La tige glisse entre ses doigts, trop mouillée. Il part ! Le basilic retombe dans l'eau, près du verre. Victorina avance les mains, trop vite. Un citron, alors ! Elle porte un citron trop près du nez. Le citron pique trop, trop acide. Il pique ! Victorina avance trop vite vers le jaune. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le citron, un instant. Elle écoute le marché, près de la barquette. Sur le plastique, un &lt;emphasis level="moderate"&gt;éclat de barquette&lt;/emphasis&gt; luit. Là, sur le plastique. Tu vois le point, Victorina ? Oui, papa. Le premier citron reste trop acide, trop près. Pas celui-là. Tu en vois un autre, Victorina ? Plus rond. Un citron plus rond attend à hauteur de main. Celui-là, maman. Tu le prends, Victorina ? Oui, papa. Victorina choisit le citron plus rond, sans se presser. La peau est lisse et froide. Il est lourd. Il tient dans ta main ? Oui, maman. Victorina le pose dans le panier. Mon citron. Il a une petite trace, Victorina. Il a failli piquer. Le citron sent le vert, un peu. Et le basilic, autour. On reste près de la barquette ? Oui.&lt;/prosody&gt;&lt;break time="420ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>Geneviève tient le citron. Maman porte le panier. [pause]</t>
+          <t>Victorina lève la main vers le basilic. Je le prends ! La tige glisse entre ses doigts, trop mouillée. Il part ! Le basilic retombe dans l'eau, près du verre. Victorina avance les mains, trop vite. Un citron, alors ! Elle porte un citron trop près du nez. Le citron pique trop, trop acide. Il pique ! Victorina avance trop vite vers le jaune. Puis elle s'arrête net. Victorina refuse de foncer, cette fois. Ses mains se ferment, puis s'ouvrent. Personne ne dit la suite. Elle observe le citron, un instant. Elle écoute le marché, près de la barquette. Sur le plastique, un &lt;emphasis&gt;éclat de barquette&lt;/emphasis&gt; luit. Là, sur le plastique. Tu vois le point, Victorina ? Oui, papa. Le premier citron reste trop acide, trop près. Pas celui-là. Tu en vois un autre, Victorina ? Plus rond. Un citron plus rond attend à hauteur de main. Celui-là, maman. Tu le prends, Victorina ? Oui, papa. Victorina choisit le citron plus rond, sans se presser. La peau est lisse et froide. Il est lourd. Il tient dans ta main ? Oui, maman. Victorina le pose dans le panier. Mon citron. Il a une petite trace, Victorina. Il a failli piquer. Le citron sent le vert, un peu. Et le basilic, autour. On reste près de la barquette ? Oui. [pause]</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr"/>
@@ -1824,7 +1879,7 @@
         </is>
       </c>
       <c r="Y5" s="2" t="n">
-        <v>132</v>
+        <v>146</v>
       </c>
       <c r="Z5" s="2" t="inlineStr">
         <is>
@@ -1832,10 +1887,10 @@
         </is>
       </c>
       <c r="AA5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AB5" s="2" t="n">
-        <v>1.18</v>
+        <v>1.1</v>
       </c>
       <c r="AC5" s="2" t="inlineStr">
         <is>
@@ -1856,28 +1911,32 @@
       <c r="AG5" s="2" t="n">
         <v>0</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr"/>
+      <c r="AH5" s="2" t="inlineStr">
+        <is>
+          <t>éclat de barquette</t>
+        </is>
+      </c>
       <c r="AI5" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ5" s="2" t="n">
-        <v>450</v>
+        <v>420</v>
       </c>
       <c r="AK5" s="2" t="n">
-        <v>280</v>
+        <v>250</v>
       </c>
       <c r="AL5" s="2" t="inlineStr">
         <is>
-          <t>calm</t>
+          <t>lively</t>
         </is>
       </c>
       <c r="AM5" s="2" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>dynamic</t>
         </is>
       </c>
       <c r="AN5" s="2" t="n">
-        <v>0.333</v>
+        <v>0.37</v>
       </c>
       <c r="AO5" s="2" t="inlineStr"/>
       <c r="AP5" s="2" t="inlineStr">
@@ -1886,10 +1945,10 @@
         </is>
       </c>
       <c r="AQ5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AR5" s="2" t="n">
-        <v>0.92</v>
+        <v>1</v>
       </c>
       <c r="AS5" s="2" t="n">
         <v>100</v>
@@ -1900,20 +1959,60 @@
       <c r="AU5" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AV5" s="2" t="inlineStr"/>
+      <c r="AV5" s="2" t="inlineStr">
+        <is>
+          <t>arc=action; intention=entraîner; emotion=élan puis prudence; intensite=2; destinataire=enfant; sous_texte=basilic_qui_glisse_citron_trop_acide_elle_choisit; tempo=vif puis posé; sourire=léger; respiration=courte</t>
+        </is>
+      </c>
       <c r="AW5" t="inlineStr">
         <is>
-          <t>narrateur|Victorina tient le citron.
-narrateur|Maman porte le panier.
-maman|On rentre tout doucement ?
+          <t>narrateur|Victorina lève la main vers le basilic.
+enfant-f|Je le prends !
+narrateur|La tige glisse entre ses doigts, trop mouillée.
+enfant-f|Il part !
+narrateur|Le basilic retombe dans l'eau, près du verre.
+narrateur|Victorina avance les mains, trop vite.
+enfant-f|Un citron, alors !
+narrateur|Elle porte un citron trop près du nez.
+narrateur|Le citron pique trop, trop acide.
+enfant-f|Il pique !
+narrateur|Victorina avance trop vite vers le jaune.
+narrateur|Puis elle s'arrête net.
+narrateur|Victorina refuse de foncer, cette fois.
+narrateur|Ses mains se ferment, puis s'ouvrent.
+narrateur|Personne ne dit la suite.
+narrateur|Elle observe le citron, un instant.
+narrateur|Elle écoute le marché, près de la barquette.
+narrateur|Sur le plastique, un éclat de barquette luit.
+enfant-f|Là, sur le plastique.
+papa|Tu vois le point, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Le premier citron reste trop acide, trop près.
+enfant-f|Pas celui-là.
+maman|Tu en vois un autre, Victorina ?
+enfant-f|Plus rond.
+narrateur|Un citron plus rond attend à hauteur de main.
+enfant-f|Celui-là, maman.
+papa|Tu le prends, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Victorina choisit le citron plus rond, sans se presser.
+narrateur|La peau est lisse et froide.
+enfant-f|Il est lourd.
+maman|Il tient dans ta main ?
 enfant-f|Oui, maman.
-maman|Tu as nommé : déçue.
-maman|Puis tu as cherché.
-narrateur|Le citron reste frais dans sa main.
-narrateur|Une feuille de basilic sent encore.
-enfant-f|Il est lisse.
-maman|Oui.
-maman|Avec l'autre idée.</t>
+narrateur|Victorina le pose dans le panier.
+enfant-f|Mon citron.
+papa|Il a une petite trace, Victorina.
+enfant-f|Il a failli piquer.
+narrateur|Le citron sent le vert, un peu.
+enfant-f|Et le basilic, autour.
+papa|On reste près de la barquette ?
+enfant-f|Oui.</t>
+        </is>
+      </c>
+      <c r="AX5" t="inlineStr">
+        <is>
+          <t>marché,citron</t>
         </is>
       </c>
     </row>
@@ -1940,17 +2039,17 @@
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Victorina. Le citron reste dans le panier.</t>
+          <t>Ils restent près de la barquette. Maman essuie un peu d'eau sur le plastique. Le citron a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Victorina tapote le plastique de la barquette. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le citron est resté, Victorina. Oui, avec nous. Le citron roule dans le panier, presque dehors. Il bascule ! Puis il tient, contre le tissu du panier. Ça sent le basilic, un peu tiède. Et le plastique, maman. Oui, dans l'air. Le marché sent les herbes, Victorina ? Oui, papa. Le citron reste contre le panier. Un éclat de barquette tient sur le plastique.</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>J'ai dit : je suis déçue. J'ai trouvé une autre idée. Bravo, Victorina. Le citron reste dans le panier.</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Ils restent près de la barquette. Maman essuie un peu d'eau sur le plastique. Le citron a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Victorina tapote le plastique de la barquette. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le citron est resté, Victorina. Oui, avec nous. Le citron roule dans le panier, presque dehors. Il bascule ! Puis il tient, contre le tissu du panier. Ça sent le basilic, un peu tiède. Et le plastique, maman. Oui, dans l'air. Le marché sent les herbes, Victorina ? Oui, papa. Le citron reste contre le panier. Un &lt;emphasis level="moderate"&gt;éclat de barquette&lt;/emphasis&gt; tient sur le plastique.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>&lt;lower-pitch&gt;&lt;soft&gt;&lt;slow&gt;L'histoire est finie.&lt;/slow&gt;&lt;/soft&gt;&lt;/lower-pitch&gt; [pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Ils restent près de la barquette. Maman essuie un peu d'eau sur le plastique. Le citron a une trace, papa. Tu l'as vue, toi ? Oui, près du bord. On est bien, ici. Victorina tapote le plastique de la barquette. Il a une trace d'eau. Tu la vois, la trace ? Oui, maman. Le citron est resté, Victorina. Oui, avec nous. Le citron roule dans le panier, presque dehors. Il bascule ! Puis il tient, contre le tissu du panier. Ça sent le basilic, un peu tiède. Et le plastique, maman. Oui, dans l'air. Le marché sent les herbes, Victorina ? Oui, papa. Le citron reste contre le panier. Un &lt;emphasis&gt;éclat de barquette&lt;/emphasis&gt; tient sur le plastique.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr"/>
@@ -1997,7 +2096,7 @@
         </is>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="Z6" s="2" t="inlineStr">
         <is>
@@ -2005,10 +2104,10 @@
         </is>
       </c>
       <c r="AA6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AB6" s="2" t="n">
-        <v>1.26</v>
+        <v>1.28</v>
       </c>
       <c r="AC6" s="2" t="inlineStr">
         <is>
@@ -2017,12 +2116,12 @@
       </c>
       <c r="AD6" s="2" t="inlineStr">
         <is>
-          <t>low</t>
+          <t>-2st</t>
         </is>
       </c>
       <c r="AE6" s="2" t="inlineStr">
         <is>
-          <t>lower-pitch</t>
+          <t>low-pitch</t>
         </is>
       </c>
       <c r="AF6" s="2" t="inlineStr">
@@ -2031,17 +2130,21 @@
         </is>
       </c>
       <c r="AG6" s="2" t="n">
-        <v>-2</v>
-      </c>
-      <c r="AH6" s="2" t="inlineStr"/>
+        <v>-3</v>
+      </c>
+      <c r="AH6" s="2" t="inlineStr">
+        <is>
+          <t>éclat de barquette</t>
+        </is>
+      </c>
       <c r="AI6" s="2" t="n">
         <v>200</v>
       </c>
       <c r="AJ6" s="2" t="n">
-        <v>600</v>
+        <v>900</v>
       </c>
       <c r="AK6" s="2" t="n">
-        <v>280</v>
+        <v>340</v>
       </c>
       <c r="AL6" s="2" t="inlineStr">
         <is>
@@ -2050,11 +2153,11 @@
       </c>
       <c r="AM6" s="2" t="inlineStr">
         <is>
-          <t>fall</t>
+          <t>falling</t>
         </is>
       </c>
       <c r="AN6" s="2" t="n">
-        <v>0.333</v>
+        <v>0.31</v>
       </c>
       <c r="AO6" s="2" t="inlineStr"/>
       <c r="AP6" s="2" t="inlineStr">
@@ -2063,27 +2166,49 @@
         </is>
       </c>
       <c r="AQ6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AR6" s="2" t="n">
-        <v>0.88</v>
+        <v>0.85</v>
       </c>
       <c r="AS6" s="2" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="AT6" s="2" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
       <c r="AU6" s="2" t="n">
-        <v>8</v>
-      </c>
-      <c r="AV6" s="2" t="inlineStr"/>
+        <v>12</v>
+      </c>
+      <c r="AV6" s="2" t="inlineStr">
+        <is>
+          <t>arc=retour; intention=refermer; emotion=tendresse_et_soulagement; intensite=1; destinataire=enfant; sous_texte=l_eclat_du_debut_tient_sur_le_plastique; tempo=posé; sourire=léger; respiration=ample</t>
+        </is>
+      </c>
       <c r="AW6" t="inlineStr">
         <is>
-          <t>enfant-f|J'ai dit : je suis déçue.
-enfant-f|J'ai trouvé une autre idée.
-maman|Bravo, Victorina.
-narrateur|Le citron reste dans le panier.</t>
+          <t>narrateur|Ils restent près de la barquette.
+narrateur|Maman essuie un peu d'eau sur le plastique.
+enfant-f|Le citron a une trace, papa.
+papa|Tu l'as vue, toi ?
+enfant-f|Oui, près du bord.
+maman|On est bien, ici.
+narrateur|Victorina tapote le plastique de la barquette.
+enfant-f|Il a une trace d'eau.
+maman|Tu la vois, la trace ?
+enfant-f|Oui, maman.
+papa|Le citron est resté, Victorina.
+enfant-f|Oui, avec nous.
+narrateur|Le citron roule dans le panier, presque dehors.
+enfant-f|Il bascule !
+narrateur|Puis il tient, contre le tissu du panier.
+narrateur|Ça sent le basilic, un peu tiède.
+enfant-f|Et le plastique, maman.
+maman|Oui, dans l'air.
+papa|Le marché sent les herbes, Victorina ?
+enfant-f|Oui, papa.
+narrateur|Le citron reste contre le panier.
+narrateur|Un éclat de barquette tient sur le plastique.</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2229,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A7"/>
+  <dimension ref="A1:A8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -2154,6 +2279,13 @@
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>